<commit_message>
docs: refresh submission artifacts
</commit_message>
<xml_diff>
--- a/docs/SIT_UAT_Test_Cases.xlsx
+++ b/docs/SIT_UAT_Test_Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R8168419449d54937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rfa8d1c933ccd4f5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -192,7 +192,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SitUatCasesTable" displayName="SitUatCasesTable" ref="A4:I14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SitUatCasesTable" displayName="SitUatCasesTable" ref="A4:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Test Case ID"/>
     <x:tableColumn id="2" name="Module"/>
@@ -445,8 +445,8 @@
         <x:v>Recorded test cases</x:v>
       </x:c>
       <x:c r="B3" s="11" t="n">
-        <x:f>COUNTA(A5:A14)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTA(A5:A15)</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
         <x:v>Source of truth</x:v>
@@ -665,28 +665,28 @@
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" s="16" t="str">
-        <x:v>UAT-001</x:v>
+        <x:v>SIT-007</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>User acceptance</x:v>
+        <x:v>Browser workflow</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>User receives a useful meeting summary</x:v>
+        <x:v>Analyze four instructor meeting-note styles</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
-        <x:v>Supported transcript available</x:v>
+        <x:v>Application is open and all four supplied TXT files are available</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>format-a.txt</x:v>
+        <x:v>English/Thai rough notes, structured follow-ups, and Thai conflict dialogue</x:v>
       </x:c>
       <x:c r="F11" s="16" t="str">
-        <x:v>Upload, analyze, review result card.</x:v>
+        <x:v>Upload all four files; analyze; navigate meetings 1 through 4; inspect evidence-bound results.</x:v>
       </x:c>
       <x:c r="G11" s="16" t="str">
-        <x:v>User can identify participants, subject summary, and assigned work.</x:v>
+        <x:v>Each card shows the verified participants, topics, decisions, actions, deadlines, and unresolved/conflict warnings.</x:v>
       </x:c>
       <x:c r="H11" s="16" t="str">
-        <x:v>e2e/meeting-analysis.spec.ts — uploads and analyzes a transcript into structured meeting results</x:v>
+        <x:v>e2e/meeting-analysis.spec.ts — renders evidence-based results for all four instructor meeting-note samples</x:v>
       </x:c>
       <x:c r="I11" s="24" t="str">
         <x:v>PASS</x:v>
@@ -694,28 +694,28 @@
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:v>UAT-002</x:v>
+        <x:v>UAT-001</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
         <x:v>User acceptance</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
-        <x:v>User identifies missing ownership</x:v>
+        <x:v>User receives a useful meeting summary</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
-        <x:v>Ownerless requirement transcript available</x:v>
+        <x:v>Supported transcript available</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>missing-owner.txt</x:v>
+        <x:v>format-a.txt</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
-        <x:v>Upload with another meeting; analyze; review owner groups.</x:v>
+        <x:v>Upload, analyze, review result card.</x:v>
       </x:c>
       <x:c r="G12" s="16" t="str">
-        <x:v>Task appears under Unassigned and is visibly warned.</x:v>
+        <x:v>User can identify participants, subject summary, and assigned work.</x:v>
       </x:c>
       <x:c r="H12" s="16" t="str">
-        <x:v>e2e/meeting-analysis.spec.ts — keeps additive upload rounds and groups actions by owner</x:v>
+        <x:v>e2e/meeting-analysis.spec.ts — uploads and analyzes a transcript into structured meeting results</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
         <x:v>PASS</x:v>
@@ -723,28 +723,28 @@
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" s="16" t="str">
-        <x:v>UAT-003</x:v>
+        <x:v>UAT-002</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
         <x:v>User acceptance</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
-        <x:v>User identifies unresolved discussion</x:v>
+        <x:v>User identifies missing ownership</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
-        <x:v>Transcript offers alternatives without resolution</x:v>
+        <x:v>Ownerless requirement transcript available</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>no-decision.txt</x:v>
+        <x:v>missing-owner.txt</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
-        <x:v>Upload; analyze; review warning.</x:v>
+        <x:v>Upload with another meeting; analyze; review owner groups.</x:v>
       </x:c>
       <x:c r="G13" s="16" t="str">
-        <x:v>User sees no-decision status without an invented outcome.</x:v>
+        <x:v>Task appears under Unassigned and is visibly warned.</x:v>
       </x:c>
       <x:c r="H13" s="16" t="str">
-        <x:v>e2e/meeting-analysis.spec.ts — shows a prominent no-decision warning without inventing a decision</x:v>
+        <x:v>e2e/meeting-analysis.spec.ts — keeps additive upload rounds and groups actions by owner</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
         <x:v>PASS</x:v>
@@ -752,30 +752,59 @@
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:v>UAT-004</x:v>
+        <x:v>UAT-003</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
         <x:v>User acceptance</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
+        <x:v>User identifies unresolved discussion</x:v>
+      </x:c>
+      <x:c r="D14" s="16" t="str">
+        <x:v>Transcript offers alternatives without resolution</x:v>
+      </x:c>
+      <x:c r="E14" s="16" t="str">
+        <x:v>no-decision.txt</x:v>
+      </x:c>
+      <x:c r="F14" s="16" t="str">
+        <x:v>Upload; analyze; review warning.</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="str">
+        <x:v>User sees no-decision status without an invented outcome.</x:v>
+      </x:c>
+      <x:c r="H14" s="16" t="str">
+        <x:v>e2e/meeting-analysis.spec.ts — shows a prominent no-decision warning without inventing a decision</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="62" customHeight="1">
+      <x:c r="A15" s="16" t="str">
+        <x:v>UAT-004</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>User acceptance</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
         <x:v>User exports analysis for sharing</x:v>
       </x:c>
-      <x:c r="D14" s="16" t="str">
+      <x:c r="D15" s="16" t="str">
         <x:v>Completed analysis</x:v>
       </x:c>
-      <x:c r="E14" s="16" t="str">
+      <x:c r="E15" s="16" t="str">
         <x:v>Analyzed meeting</x:v>
       </x:c>
-      <x:c r="F14" s="16" t="str">
+      <x:c r="F15" s="16" t="str">
         <x:v>Click Download Word Report; open the file.</x:v>
       </x:c>
-      <x:c r="G14" s="16" t="str">
+      <x:c r="G15" s="16" t="str">
         <x:v>Readable report contains the analyzed meeting and grouped actions.</x:v>
       </x:c>
-      <x:c r="H14" s="16" t="str">
+      <x:c r="H15" s="16" t="str">
         <x:v>e2e/meeting-analysis.spec.ts — downloads a structurally recognizable Word report</x:v>
       </x:c>
-      <x:c r="I14" s="24" t="str">
+      <x:c r="I15" s="24" t="str">
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
@@ -787,7 +816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fbaee17e76b451b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc6eebfe34b649e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>